<commit_message>
Add SEO batch 1: Brighton, letterbox drop cost, Local Businesses, Home Services, Plumbers
- New landing pages built from docs/seo/sef-page-build-context.md
- Shared landing components (hero, proof strip, sections, CTA)
- Home Services hub replaces Trades & Services (308 redirect)
- FAQ answers now in page HTML so they match FAQPage schema
- Nav, footer, industries index, Melbourne page and sitemap link the new pages
- Melbourne pricing FAQ updated to $200 per 1,000

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019SU6K2A2oyMFdSUg8CR5LM
</commit_message>
<xml_diff>
--- a/docs/seo/SEF_SEO_Page_Plan.xlsx
+++ b/docs/seo/SEF_SEO_Page_Plan.xlsx
@@ -8,15 +8,17 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Page Plan" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keyword Data" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitor - LBD" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Images" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keyword Data" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitor - LBD" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Page Plan'!$A$1:$K$81</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Keyword Data'!$A$1:$D$139</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Notes'!$A$1:$B$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Competitor - LBD'!$A$1:$C$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Images'!$A$1:$I$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Keyword Data'!$A$1:$D$139</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Notes'!$A$1:$B$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Competitor - LBD'!$A$1:$C$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -102,7 +104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -118,6 +120,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4969,6 +4974,1429 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Page</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Image type</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>File name</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>Description (brief for photographer / designer)</t>
+        </is>
+      </c>
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>Alt text</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>Size</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Local Businesses (hub)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>/industries/local-businesses</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Hero (real photo)</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>local-business-flyer-distribution-melbourne.webp</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Wide shot of two SEF walkers on a suburban street with a row of local shops behind them (cafe, barber, hardware). One is placing a flyer in a house letterbox across the road. Morning light, SEF branded tops visible, no shop logos readable.</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>South East Flyers walkers delivering flyers near a strip of local shops in Melbourne</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>1600×900 hero (crop 1200×630 for social share)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Home Services (hub)</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>/industries/home-services</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Hero (real photo)</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>home-services-letterbox-drop-melbourne.webp</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Walker delivering to a weatherboard house with a tradie's ute parked in the driveway (no signage readable). Shows the link between home owners and trades.</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Flyer being delivered to a house with a tradie ute in the driveway</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>1600×900 hero (crop 1200×630 for social share)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>/industries/real-estate</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Hero (real photo)</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>real-estate-letterbox-drop.webp</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Walker delivering to a period home on a tree-lined street, a generic 'For Sale' board (no agency branding) on a neighbouring property.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Real estate flyer delivered to a letterbox next to a For Sale sign</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>1600×900 hero (crop 1200×630 for social share)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>/industries/real-estate</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Flyer sample (AI or designed OK)</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>just-sold-flyer-sample.webp</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>A5 'Just Sold' flyer for a fictional agency: property photo, sold price placeholder, '3 bed 2 bath', agent headshot silhouette, 'Thinking of selling? Free appraisal' call to action.</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Sample Just Sold real estate flyer</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>1200×900</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Plumbers</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>/industries/plumbers</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Hero (real photo)</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>plumber-flyer-letterbox-drop.webp</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Close-up of a hand placing a plumbing flyer into a brick-pillar letterbox; flyer visible enough to read 'Blocked drains?'.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Plumbing flyer being placed in a brick letterbox</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>1600×900 hero (crop 1200×630 for social share)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Plumbers</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>/industries/plumbers</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Flyer sample (AI or designed OK)</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>plumber-flyer-sample.webp</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>DL flyer for a fictional plumber: 'Blocked drains? Hot water out?', 24/7 call-out line, licence number placeholder, fridge-magnet tear-off strip.</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Sample plumber flyer with emergency call-out offer</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>1200×900</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Electricians</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>/industries/electricians</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Hero (real photo)</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>electrician-flyer-letterbox-drop.webp</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Walker at a modern townhouse letterbox; solar panels visible on the roof behind.</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Electrician flyer delivered to a townhouse with solar panels</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>1600×900 hero (crop 1200×630 for social share)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Electricians</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>/industries/electricians</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Flyer sample (AI or designed OK)</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>electrician-flyer-sample.webp</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>DL flyer for a fictional electrician: 'Safety switch check from $X', 'Switchboard upgrades', 'Free quote', REC number placeholder.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Sample electrician flyer for safety switch checks</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>1200×900</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Roofers</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>/industries/roofing</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Hero (real photo)</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>roofing-flyer-letterbox-drop.webp</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Walker delivering on a street of older tiled-roof homes; one roof visibly weathered. Overcast sky (storm season feel).</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Roofing flyer delivered on a street of tiled-roof homes</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>1600×900 hero (crop 1200×630 for social share)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Roofers</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>/industries/roofing</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Flyer sample (AI or designed OK)</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>roofing-flyer-sample.webp</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>A5 flyer for a fictional roofer: before/after roof restoration photos, 'Free roof inspection', 'Storm damage repairs'.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Sample roofing flyer with before and after roof restoration</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>1200×900</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Builders</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>/industries/builders</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Hero (real photo)</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>builder-flyer-letterbox-drop.webp</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Walker delivering to homes next to a construction site with scaffolding (no builder branding readable).</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Flyer delivery next to a home construction site in Melbourne</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>1600×900 hero (crop 1200×630 for social share)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Builders</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>/industries/builders</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Flyer sample (AI or designed OK)</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>builder-flyer-sample.webp</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>A5 flyer for a fictional builder: 'Knockdown rebuild specialists', render of a double-storey home, 'Free site assessment'.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Sample builder flyer for knockdown rebuild</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>1200×900</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Renovation</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>/industries/renovation</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Hero (real photo)</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>renovation-flyer-letterbox-drop.webp</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Walker at the letterbox of a 1970s brick home that is an obvious renovation candidate.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Renovation flyer delivered to an older brick home</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>1600×900 hero (crop 1200×630 for social share)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Renovation</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>/industries/renovation</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Flyer sample (AI or designed OK)</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>renovation-flyer-sample.webp</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>A5 flyer for a fictional renovator: split before/after kitchen and bathroom photos, 'Bathroom renovations from $X', 'Free design consult'.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Sample renovation flyer with bathroom before and after</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>1200×900</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Cleaning (house &amp; bathroom)</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>/industries/cleaning</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Hero (real photo)</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>house-cleaning-flyer-letterbox-drop.webp</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Walker delivering to an apartment-style townhouse block's individual letterboxes; tidy, bright setting.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>House cleaning flyer delivered to townhouse letterboxes</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>1600×900 hero (crop 1200×630 for social share)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Cleaning (house &amp; bathroom)</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>/industries/cleaning</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Flyer sample (AI or designed OK)</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>cleaning-flyer-sample.webp</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>DL flyer for a fictional cleaner: 'Regular home cleans', 'Bathroom deep clean', 'First clean 20% off', fully insured badge.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Sample house and bathroom cleaning flyer</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>1200×900</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Dog Groomers &amp; Dog Wash</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>/industries/pet-groomers</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Hero (real photo)</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>dog-grooming-flyer-letterbox-drop.webp</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Walker delivering a flyer while a friendly dog watches from behind a front gate.</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Dog grooming flyer delivered to a home with a dog at the gate</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>1600×900 hero (crop 1200×630 for social share)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Dog Groomers &amp; Dog Wash</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>/industries/pet-groomers</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Flyer sample (AI or designed OK)</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>dog-grooming-flyer-sample.webp</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>DL flyer for a fictional dog groomer / dog wash: freshly groomed dog photo, 'Mobile grooming - we come to you', 'Self-serve dog wash', first-visit offer.</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Sample dog grooming and dog wash flyer</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>1200×900</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Restaurants &amp; Cafes</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>/industries/restaurants</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Hero (real photo)</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>restaurant-menu-flyer-delivery.webp</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Walker delivering a takeaway menu flyer at dusk, warm streetlight; suburban street.</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Takeaway menu flyer delivered to a letterbox in the evening</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>1600×900 hero (crop 1200×630 for social share)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Restaurants &amp; Cafes</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>/industries/restaurants</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Flyer sample (AI or designed OK)</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>takeaway-menu-flyer-sample.webp</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Folded takeaway menu for a fictional local restaurant: food photos, menu sections, 'Order online' QR code, 'Free delivery over $40'.</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Sample takeaway menu flyer</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>1200×900</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Carpenters</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>/industries/carpenters</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Hero (real photo)</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>carpentry-flyer-letterbox-drop.webp</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Walker delivering to a house with a new timber deck and pergola visible in the front yard.</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Carpentry flyer delivered to a home with a timber deck</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>1600×900 hero (crop 1200×630 for social share)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Carpenters</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>/industries/carpenters</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Flyer sample (AI or designed OK)</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>carpentry-flyer-sample.webp</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>DL flyer for a fictional carpenter: decking, pergolas, built-in wardrobes photos, 'Free measure and quote'.</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Sample carpentry flyer for decks and pergolas</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>1200×900</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Dentists</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>/industries/dentists</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Hero (real photo)</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>dental-flyer-letterbox-drop.webp</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Walker delivering on a family street; school bag and bike near the front porch (family audience).</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Dental clinic flyer delivered to a family home</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>1600×900 hero (crop 1200×630 for social share)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Dentists</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>/industries/dentists</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Flyer sample (AI or designed OK)</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>dental-flyer-sample.webp</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>A5 flyer for a fictional dental clinic: 'New patients welcome', 'Check-up and clean', health fund logos as generic icons only, opening hours.</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Sample dental clinic new patient flyer</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>1200×900</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Vets</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>/industries/vets</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Hero (real photo)</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>vet-clinic-flyer-letterbox-drop.webp</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Walker delivering while a cat sits on the fence or a dog looks out the window.</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Vet clinic flyer delivered to a pet owner's home</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>1600×900 hero (crop 1200×630 for social share)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Vets</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>/industries/vets</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Flyer sample (AI or designed OK)</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>vet-flyer-sample.webp</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>A5 flyer for a fictional vet: 'Puppy and kitten vaccination packages', 'Dental month', clinic hours, map snippet.</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Sample vet clinic flyer for vaccinations</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>1200×900</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>GPs &amp; Medical Clinics</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>/industries/medical-clinics</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Hero (real photo)</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>medical-clinic-flyer-letterbox-drop.webp</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Walker delivering on a street of mixed homes and units; mid-morning, neutral and calm.</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Medical clinic flyer delivered to a letterbox</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>1600×900 hero (crop 1200×630 for social share)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>GPs &amp; Medical Clinics</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>/industries/medical-clinics</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Flyer sample (AI or designed OK)</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>medical-clinic-flyer-sample.webp</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>A5 flyer for a fictional GP clinic: 'Now open', 'Bulk billing available', doctors' specialties, opening hours. No health claims.</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Sample medical clinic opening flyer</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>1200×900</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Schools &amp; Childcare</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>/industries/schools-childcare</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Hero (real photo)</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>childcare-enrolment-flyer-delivery.webp</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Walker delivering on a family street near a park or playground.</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Childcare enrolment flyer delivered near a local park</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>1600×900 hero (crop 1200×630 for social share)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Schools &amp; Childcare</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>/industries/schools-childcare</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Flyer sample (AI or designed OK)</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>childcare-enrolment-flyer-sample.webp</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>A5 flyer for a fictional childcare centre: 'Enrolments open for 2027', 'Book a tour', bright play area photo (no identifiable children).</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Sample childcare enrolment flyer</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>1200×900</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I31"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -8042,7 +9470,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8169,7 +9597,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>